<commit_message>
implementation of wordtemplateprocessor, created true template for earnings report template, added SM lung transplant workbook
</commit_message>
<xml_diff>
--- a/EconAutomation/src/supporting_docs/sorted_econ_files/2PV_Annual_temp_new (color coded).xlsx
+++ b/EconAutomation/src/supporting_docs/sorted_econ_files/2PV_Annual_temp_new (color coded).xlsx
@@ -6,12 +6,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\EricBussey\GitHub\Stokes-Scripts\EconAutomation\src\supporting_docs\sorted_econ_files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\EricBussey\GitHub\EconAutomation-REP\EconAutomation\src\supporting_docs\sorted_econ_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="8_{5FFE6F5C-450D-4611-AF89-06C9F991CA2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-60" windowWidth="29040" windowHeight="15720" activeTab="17" xr2:uid="{25EC3B8A-402B-47FF-80A9-5B0690A475CD}"/>
+    <workbookView xWindow="28680" yWindow="-60" windowWidth="29040" windowHeight="15720" xr2:uid="{25EC3B8A-402B-47FF-80A9-5B0690A475CD}"/>
   </bookViews>
   <sheets>
     <sheet name="Case Inputs" sheetId="3" r:id="rId1"/>
@@ -3629,7 +3629,7 @@
     <mergeCell ref="A26:D26"/>
   </mergeCells>
   <phoneticPr fontId="0" type="noConversion"/>
-  <dataValidations count="2">
+  <dataValidations disablePrompts="1" count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B28" xr:uid="{538D03BE-50D6-475B-B155-93A8C8C6ED02}">
       <formula1>"CPI Adjustment,No Adjustment,Custom Rate"</formula1>
     </dataValidation>

</xml_diff>